<commit_message>
feat: add import functionality for Employees and Roles with UI components
- Introduced MasterImportAction and MasterImportDialog components for handling file uploads.
- Implemented import logic for Employees and Roles, including error reporting and success messages.
- Created MasterStatusChips and useStatusCounts hooks to display and manage status counts for master records.
- Added Excel file templates for Employees and Roles import.
</commit_message>
<xml_diff>
--- a/docs/import/Suppliers.xlsx
+++ b/docs/import/Suppliers.xlsx
@@ -3376,8 +3376,10 @@
       <x:c r="AJ15" s="0" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="AK15" s="0" t="s">
-        <x:v>315</x:v>
+      <x:c r="AK15" s="0" t="inlineStr">
+        <x:is>
+          <x:t>Hold</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:37">

</xml_diff>